<commit_message>
Update research papers spreadsheet after third search round
Confirm authors for the TLBO-SGO clustering paper (#20) and add the
Springer conference paper listed in the PBAS form.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PzLbErSZvTchNCi41JwS9b
</commit_message>
<xml_diff>
--- a/Available_Research_Papers.xlsx
+++ b/Available_Research_Papers.xlsx
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -105,6 +105,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -182,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Papers" displayName="Papers" ref="A1:H13" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Papers" displayName="Papers" ref="A1:H14" headerRowCount="1">
   <autoFilter ref="A1:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="PBAS #"/>
@@ -487,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -969,7 +972,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Kanaka Raghu Sreerama et al.</t>
+          <t>Kanaka Raghu Sreerama, M. Ramakrishna Murthy, K. Venkata Ramana</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -984,46 +987,85 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Probable match</t>
+          <t>Citation only</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Work is part of Kanaka Raghu Sreerama's thesis; journal publication not confirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+          <t>Authors confirmed by search snippet; no direct URL found. Proposes ITLBOSGOTEA and ITLBOSGOPEA hybrid algorithms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Conf. 1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Secured Surveillance Storage Model Using Blockchain</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>D. Soujanya, K. Venkata Ramana</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Evolving Technologies for Computing, Communication and Smart World (Springer), pp. 249–263, 2021</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Springer (conference)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Citation only</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Listed under 'Publications Other than Journal Articles' in the PBAS form, not among the 26 journal papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Source: PBAS application PBAS-202693-13299 (26 listed journal papers); web searches run 2026-09-29.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>DOIs for #7, #9, #14 are taken from the PBAS form; doi.org links were not opened (blocked from the search environment).</t>
+          <t>Source: PBAS application PBAS-202693-13299 (26 listed journal papers); web searches run 2026-09-29 (three rounds).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>14 other listed titles (#1, 2, 3, 5, 6, 8, 12, 13, 15, 17, 18, 21, 25, 26) could not be found online and are not included.</t>
+          <t>DOIs for #7, #9, #14 are taken from the PBAS form; doi.org links were not opened (blocked from the search environment).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>14 listed journal titles (#1, 2, 3, 5, 6, 8, 12, 13, 15, 17, 18, 21, 25, 26) could not be found online and are not included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>#26's title is identical to Han et al., IEEE Trans. Dependable &amp; Secure Computing 2019 (different authors) — worth verifying.</t>
         </is>

</xml_diff>